<commit_message>
Latest code added for France
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataFranceMK.xlsx
+++ b/Data/Hires/TestDataFranceMK.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="283">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -229,7 +229,7 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10698370</t>
+    <t>10698400</t>
   </si>
   <si>
     <t>Passed</t>
@@ -244,10 +244,10 @@
     <t>Madame</t>
   </si>
   <si>
-    <t>Kiarra</t>
-  </si>
-  <si>
-    <t>Funk</t>
+    <t>Delphine</t>
+  </si>
+  <si>
+    <t>Davis-Kling</t>
   </si>
   <si>
     <t>03 48 29 85 70</t>
@@ -382,19 +382,19 @@
     <t>Test3</t>
   </si>
   <si>
-    <t>10698371</t>
+    <t>10698401</t>
   </si>
   <si>
     <t>221 Store Management (Pucyw Zipato (9221018))</t>
   </si>
   <si>
-    <t>Isaiah</t>
-  </si>
-  <si>
-    <t>Lebsack</t>
-  </si>
-  <si>
-    <t>Auto 29786886</t>
+    <t>Duane</t>
+  </si>
+  <si>
+    <t>Emmerich</t>
+  </si>
+  <si>
+    <t>Auto 5320099</t>
   </si>
   <si>
     <t>Store Manager</t>
@@ -424,16 +424,378 @@
     <t>Test4</t>
   </si>
   <si>
-    <t>10698359</t>
-  </si>
-  <si>
-    <t>Emmett</t>
-  </si>
-  <si>
-    <t>Gutmann</t>
-  </si>
-  <si>
-    <t>Auto 97380354</t>
+    <t xml:space="preserve">Test failed for 'Renee Lang' Employee:{10698402}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for locator('//div[@data-automation-id="tooltipsWrapper"]/button[@data-automation-id="inbox_preview"]').first()[22m
+[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #1[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #2[22m
+[2m  -   waiting 20ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #3[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #4[22m
+[2m  -   waiting 100ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #5[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #6[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #7[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #8[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #9[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #10[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #11[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #12[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #13[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #14[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #15[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #16[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #17[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #18[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #19[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #20[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #21[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #22[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #23[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #24[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #25[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #26[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #27[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #28[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #29[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #30[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #31[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #32[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #33[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #34[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #35[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #36[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #37[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #38[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #39[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #40[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #41[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #42[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #43[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #44[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #45[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #46[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #47[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #48[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #49[22m
+[2m  -   waiting 500ms[22m
+[2m  -   waiting for element to be visible, enabled and stable[22m
+[2m  -   element is visible, enabled and stable[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+[2m  -   &lt;div role="none" class="css-1jo90af"&gt;…&lt;/div&gt; from &lt;section aria-live="polite" aria-label="Notifications"&gt;…&lt;/section&gt; subtree intercepts pointer events[22m
+[2m  - retrying click action, attempt #50[22m
+[2m  -   waiting 500ms[22m
+</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Renee</t>
+  </si>
+  <si>
+    <t>Lang</t>
+  </si>
+  <si>
+    <t>Auto 28725953</t>
   </si>
   <si>
     <t>Department Manager</t>
@@ -445,16 +807,13 @@
     <t>Test5</t>
   </si>
   <si>
-    <t>10698362</t>
-  </si>
-  <si>
-    <t>Chelsie</t>
-  </si>
-  <si>
-    <t>Toy</t>
-  </si>
-  <si>
-    <t>Auto 91674261</t>
+    <t>Bailee</t>
+  </si>
+  <si>
+    <t>Kunze</t>
+  </si>
+  <si>
+    <t>Auto 34305455</t>
   </si>
   <si>
     <t>Fixed Term (Fixed Term)</t>
@@ -487,16 +846,16 @@
     <t>Test6</t>
   </si>
   <si>
-    <t>10698365</t>
-  </si>
-  <si>
-    <t>Rachael</t>
-  </si>
-  <si>
-    <t>Jerde-Kuphal</t>
-  </si>
-  <si>
-    <t>Auto 96494734</t>
+    <t>10698403</t>
+  </si>
+  <si>
+    <t>Korbin</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>Auto 94727550</t>
   </si>
   <si>
     <t>Trainee Manager</t>
@@ -511,19 +870,19 @@
     <t>Test7</t>
   </si>
   <si>
-    <t>10698368</t>
-  </si>
-  <si>
-    <t>Estel</t>
-  </si>
-  <si>
-    <t>Kessler</t>
+    <t>10698404</t>
+  </si>
+  <si>
+    <t>Krystal</t>
+  </si>
+  <si>
+    <t>Sipes</t>
   </si>
   <si>
     <t>4 48 29 85 70</t>
   </si>
   <si>
-    <t>Auto 98018235</t>
+    <t>Auto 53957765</t>
   </si>
   <si>
     <t>Assistant Manager</t>
@@ -535,6 +894,15 @@
     <t>Test8</t>
   </si>
   <si>
+    <t>10698405</t>
+  </si>
+  <si>
+    <t>Ocie</t>
+  </si>
+  <si>
+    <t>Macejkovic</t>
+  </si>
+  <si>
     <t>5 48 29 85 70</t>
   </si>
   <si>
@@ -556,9 +924,21 @@
     <t>Test9</t>
   </si>
   <si>
+    <t xml:space="preserve">Test failed for 'Crystel Schinner' Employee:{}TimeoutError: locator.focus: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByLabel('Position Request Reason')[22m
+</t>
+  </si>
+  <si>
     <t>221 Store Management (Rykil Wuhoga (9221018))</t>
   </si>
   <si>
+    <t>Crystel</t>
+  </si>
+  <si>
+    <t>Schinner</t>
+  </si>
+  <si>
     <t>6 48 29 85 70</t>
   </si>
   <si>
@@ -574,6 +954,15 @@
     <t>Test10</t>
   </si>
   <si>
+    <t>10698406</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Krajcik</t>
+  </si>
+  <si>
     <t>7 48 29 85 70</t>
   </si>
   <si>
@@ -583,6 +972,15 @@
     <t>Test11</t>
   </si>
   <si>
+    <t>10698407</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Vandervort</t>
+  </si>
+  <si>
     <t>Supervisor</t>
   </si>
   <si>
@@ -598,12 +996,30 @@
     <t>Test12</t>
   </si>
   <si>
+    <t>10698408</t>
+  </si>
+  <si>
+    <t>Lester</t>
+  </si>
+  <si>
+    <t>Nicolas</t>
+  </si>
+  <si>
     <t>P&amp;C Supervisor (NLD/FRA/USA/ITA/PL/CZ ONLY)</t>
   </si>
   <si>
     <t>Test13</t>
   </si>
   <si>
+    <t>10698409</t>
+  </si>
+  <si>
+    <t>Dedrick</t>
+  </si>
+  <si>
+    <t>Turcotte</t>
+  </si>
+  <si>
     <t>Contrat apprentissage</t>
   </si>
   <si>
@@ -634,6 +1050,15 @@
     <t>Test14</t>
   </si>
   <si>
+    <t>10698410</t>
+  </si>
+  <si>
+    <t>Meghan</t>
+  </si>
+  <si>
+    <t>Thiel</t>
+  </si>
+  <si>
     <t>Visuel Merchandiser</t>
   </si>
   <si>
@@ -652,19 +1077,154 @@
     <t>Test15</t>
   </si>
   <si>
+    <t>10698411</t>
+  </si>
+  <si>
+    <t>Sadye</t>
+  </si>
+  <si>
+    <t>Durgan</t>
+  </si>
+  <si>
     <t>08 Ladieswear</t>
   </si>
   <si>
     <t>Test16</t>
   </si>
   <si>
+    <t>10698412</t>
+  </si>
+  <si>
+    <t>Cyrus</t>
+  </si>
+  <si>
+    <t>Kihn</t>
+  </si>
+  <si>
     <t>05 Childrens Wear</t>
   </si>
   <si>
+    <t>Test failed for 'Manley Ward' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Reyes</t>
+  </si>
+  <si>
+    <t>Douglas</t>
+  </si>
+  <si>
+    <t>Test failed for 'Alicia Conroy' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Test failed for 'Paris Paucek' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Test failed for 'Evalyn Hauck' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Tomas</t>
+  </si>
+  <si>
+    <t>Borer</t>
+  </si>
+  <si>
+    <t>Test failed for 'Malvina Kessler' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Magali</t>
+  </si>
+  <si>
+    <t>Abbott</t>
+  </si>
+  <si>
+    <t>Test failed for 'Isabell Wolff' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Marshall</t>
+  </si>
+  <si>
+    <t>Johns</t>
+  </si>
+  <si>
+    <t>Angus</t>
+  </si>
+  <si>
+    <t>Tillman</t>
+  </si>
+  <si>
+    <t>Test failed for 'Andres Herzog' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
     <t>X</t>
   </si>
   <si>
-    <t>RRBABA</t>
+    <t>RSBABA</t>
+  </si>
+  <si>
+    <t>Kariane</t>
+  </si>
+  <si>
+    <t>Pacocha</t>
+  </si>
+  <si>
+    <t>Test failed for 'Marianna Walker' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Test failed for 'Wyman Sauer' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Test failed for 'Dimitri Marks' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Test failed for 'Jane Stoltenberg' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Allison</t>
+  </si>
+  <si>
+    <t>Crona</t>
+  </si>
+  <si>
+    <t>Wilfrid</t>
+  </si>
+  <si>
+    <t>Spencer</t>
+  </si>
+  <si>
+    <t>Mohammed</t>
+  </si>
+  <si>
+    <t>Rodriguez</t>
+  </si>
+  <si>
+    <t>Kaelyn</t>
+  </si>
+  <si>
+    <t>Blick</t>
+  </si>
+  <si>
+    <t>Test failed for 'Deja Metz' Employee:{}TypeError: Cannot read properties of null (reading 'toString')</t>
+  </si>
+  <si>
+    <t>Victor</t>
+  </si>
+  <si>
+    <t>Stroman</t>
+  </si>
+  <si>
+    <t>Collin</t>
+  </si>
+  <si>
+    <t>Feest</t>
+  </si>
+  <si>
+    <t>Jaiden</t>
+  </si>
+  <si>
+    <t>Lesch</t>
+  </si>
+  <si>
+    <t>Test failed for 'Jalen Schulist' Employee:{undefined}TypeError: Cannot read properties of null (reading 'toString')</t>
   </si>
 </sst>
 </file>
@@ -731,7 +1291,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -765,6 +1325,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -814,7 +1379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -916,6 +1481,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1550,7 +2118,7 @@
       </c>
       <c r="L2" s="17">
         <f t="shared" ref="L2:L16" si="0">TODAY()-31</f>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M2" s="11" t="s">
         <v>74</v>
@@ -1581,7 +2149,7 @@
       </c>
       <c r="V2" s="17">
         <f t="shared" ref="V2:V16" si="1">L2</f>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W2" s="16" t="s">
         <v>87</v>
@@ -1627,15 +2195,15 @@
       </c>
       <c r="AK2" s="24">
         <f t="shared" ref="AK2:AK16" si="2">V2</f>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL2" s="24">
         <f t="shared" ref="AL2:AL16" si="3">V2</f>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM2" s="24">
         <f t="shared" ref="AM2:AM16" si="4">V2</f>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN2" s="17">
         <f t="shared" ref="AN2:AN16" si="5">AG2</f>
@@ -1664,7 +2232,7 @@
       </c>
       <c r="AV2" s="24">
         <f t="shared" ref="AV2:AV16" si="6">TODAY()+20</f>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW2" s="11" t="s">
         <v>74</v>
@@ -1674,7 +2242,7 @@
       </c>
       <c r="AY2" s="26" t="str">
         <f>BB28</f>
-        <v>X6RRBABA21</v>
+        <v>X1RSBABA18</v>
       </c>
       <c r="AZ2" s="24" t="s">
         <v>108</v>
@@ -1744,7 +2312,7 @@
       </c>
       <c r="BV2" s="31">
         <f t="array" ref="BV2:BV16">_xlfn.RANDARRAY(15,1,12345,99999,TRUE)</f>
-        <v>28402</v>
+        <v>29066</v>
       </c>
       <c r="BW2" s="24">
         <v>44562</v>
@@ -1792,7 +2360,7 @@
       </c>
       <c r="L3" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M3" s="11" t="s">
         <v>74</v>
@@ -1823,7 +2391,7 @@
       </c>
       <c r="V3" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W3" s="16" t="s">
         <v>87</v>
@@ -1869,15 +2437,15 @@
       </c>
       <c r="AK3" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL3" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM3" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN3" s="17">
         <f t="shared" si="5"/>
@@ -1906,7 +2474,7 @@
       </c>
       <c r="AV3" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW3" s="11" t="s">
         <v>74</v>
@@ -1916,7 +2484,7 @@
       </c>
       <c r="AY3" s="26" t="str">
         <f t="shared" ref="AY3:AY16" si="7">BB29</f>
-        <v>X2RRBABA34</v>
+        <v>X5RSBABA47</v>
       </c>
       <c r="AZ3" s="24" t="s">
         <v>108</v>
@@ -1985,7 +2553,7 @@
         <v>119</v>
       </c>
       <c r="BV3" s="31">
-        <v>15465</v>
+        <v>42767</v>
       </c>
       <c r="BW3" s="24">
         <v>44562</v>
@@ -2005,7 +2573,7 @@
         <v>136</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>123</v>
@@ -2017,10 +2585,10 @@
         <v>75</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I4" s="15" t="s">
         <v>78</v>
@@ -2033,7 +2601,7 @@
       </c>
       <c r="L4" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>74</v>
@@ -2064,19 +2632,19 @@
       </c>
       <c r="V4" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W4" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X4" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="Y4" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="AA4" s="12" t="s">
         <v>91</v>
@@ -2110,15 +2678,15 @@
       </c>
       <c r="AK4" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL4" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM4" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN4" s="17">
         <f t="shared" si="5"/>
@@ -2140,14 +2708,14 @@
         <v>104</v>
       </c>
       <c r="AT4" s="11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="AU4" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV4" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW4" s="11" t="s">
         <v>74</v>
@@ -2157,7 +2725,7 @@
       </c>
       <c r="AY4" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X2RRBABA36</v>
+        <v>X3RSBABA79</v>
       </c>
       <c r="AZ4" s="24" t="s">
         <v>108</v>
@@ -2226,7 +2794,7 @@
         <v>119</v>
       </c>
       <c r="BV4" s="31">
-        <v>48016</v>
+        <v>35746</v>
       </c>
       <c r="BW4" s="24">
         <v>44562</v>
@@ -2240,14 +2808,9 @@
     </row>
     <row r="5" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="B5" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C5" s="9" t="s">
-        <v>72</v>
-      </c>
+      <c r="C5" s="9"/>
       <c r="D5" s="10" t="s">
         <v>123</v>
       </c>
@@ -2274,7 +2837,7 @@
       </c>
       <c r="L5" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>74</v>
@@ -2305,7 +2868,7 @@
       </c>
       <c r="V5" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W5" s="16" t="s">
         <v>87</v>
@@ -2339,7 +2902,7 @@
       </c>
       <c r="AG5" s="23">
         <f>V5+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH5" s="16" t="s">
         <v>150</v>
@@ -2352,19 +2915,19 @@
       </c>
       <c r="AK5" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL5" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM5" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN5" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO5" s="16" t="s">
         <v>129</v>
@@ -2389,7 +2952,7 @@
       </c>
       <c r="AV5" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW5" s="11" t="s">
         <v>74</v>
@@ -2399,7 +2962,7 @@
       </c>
       <c r="AY5" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X3RRBABA41</v>
+        <v>X7RSBABA2</v>
       </c>
       <c r="AZ5" s="24" t="s">
         <v>108</v>
@@ -2468,7 +3031,7 @@
         <v>119</v>
       </c>
       <c r="BV5" s="31">
-        <v>69037</v>
+        <v>21861</v>
       </c>
       <c r="BW5" s="24">
         <v>44562</v>
@@ -2516,7 +3079,7 @@
       </c>
       <c r="L6" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M6" s="11" t="s">
         <v>74</v>
@@ -2547,7 +3110,7 @@
       </c>
       <c r="V6" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>87</v>
@@ -2593,15 +3156,15 @@
       </c>
       <c r="AK6" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL6" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM6" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN6" s="17">
         <f t="shared" si="5"/>
@@ -2630,7 +3193,7 @@
       </c>
       <c r="AV6" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW6" s="11" t="s">
         <v>74</v>
@@ -2640,7 +3203,7 @@
       </c>
       <c r="AY6" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X5RRBABA26</v>
+        <v>X3RSBABA91</v>
       </c>
       <c r="AZ6" s="24" t="s">
         <v>108</v>
@@ -2709,7 +3272,7 @@
         <v>119</v>
       </c>
       <c r="BV6" s="31">
-        <v>12863</v>
+        <v>63567</v>
       </c>
       <c r="BW6" s="24">
         <v>44562</v>
@@ -2757,7 +3320,7 @@
       </c>
       <c r="L7" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M7" s="11" t="s">
         <v>74</v>
@@ -2788,7 +3351,7 @@
       </c>
       <c r="V7" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W7" s="16" t="s">
         <v>87</v>
@@ -2834,15 +3397,15 @@
       </c>
       <c r="AK7" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL7" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM7" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN7" s="17">
         <f t="shared" si="5"/>
@@ -2871,7 +3434,7 @@
       </c>
       <c r="AV7" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW7" s="11" t="s">
         <v>74</v>
@@ -2881,7 +3444,7 @@
       </c>
       <c r="AY7" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X4RRBABA70</v>
+        <v>X8RSBABA76</v>
       </c>
       <c r="AZ7" s="24" t="s">
         <v>108</v>
@@ -2950,7 +3513,7 @@
         <v>119</v>
       </c>
       <c r="BV7" s="31">
-        <v>56785</v>
+        <v>76923</v>
       </c>
       <c r="BW7" s="24">
         <v>44562</v>
@@ -2966,8 +3529,12 @@
       <c r="A8" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
+      <c r="B8" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D8" s="10" t="s">
         <v>73</v>
       </c>
@@ -2977,10 +3544,14 @@
       <c r="F8" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="13"/>
-      <c r="H8" s="14"/>
+      <c r="G8" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="I8" s="15" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>79</v>
@@ -2990,7 +3561,7 @@
       </c>
       <c r="L8" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M8" s="11" t="s">
         <v>74</v>
@@ -3021,7 +3592,7 @@
       </c>
       <c r="V8" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W8" s="16" t="s">
         <v>87</v>
@@ -3033,7 +3604,7 @@
         <v>147</v>
       </c>
       <c r="Z8" s="12" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="AA8" s="12" t="s">
         <v>149</v>
@@ -3055,7 +3626,7 @@
       </c>
       <c r="AG8" s="23">
         <f>V8+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH8" s="16" t="s">
         <v>150</v>
@@ -3068,44 +3639,44 @@
       </c>
       <c r="AK8" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL8" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM8" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN8" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO8" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP8" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AQ8" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR8" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AS8" s="16" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AT8" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AU8" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV8" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW8" s="11" t="s">
         <v>74</v>
@@ -3115,7 +3686,7 @@
       </c>
       <c r="AY8" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X7RRBABA41</v>
+        <v>X1RSBABA81</v>
       </c>
       <c r="AZ8" s="24" t="s">
         <v>108</v>
@@ -3184,7 +3755,7 @@
         <v>119</v>
       </c>
       <c r="BV8" s="31">
-        <v>15562</v>
+        <v>48339</v>
       </c>
       <c r="BW8" s="24">
         <v>44562</v>
@@ -3198,11 +3769,16 @@
     </row>
     <row r="9" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="C9" s="9"/>
+        <v>182</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>137</v>
+      </c>
       <c r="D9" s="10" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>74</v>
@@ -3210,10 +3786,14 @@
       <c r="F9" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="14"/>
+      <c r="G9" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>186</v>
+      </c>
       <c r="I9" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J9" s="16" t="s">
         <v>79</v>
@@ -3223,7 +3803,7 @@
       </c>
       <c r="L9" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M9" s="11" t="s">
         <v>74</v>
@@ -3254,19 +3834,19 @@
       </c>
       <c r="V9" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X9" s="13" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="Y9" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="AA9" s="12" t="s">
         <v>91</v>
@@ -3300,15 +3880,15 @@
       </c>
       <c r="AK9" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL9" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM9" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN9" s="17">
         <f t="shared" si="5"/>
@@ -3330,14 +3910,14 @@
         <v>152</v>
       </c>
       <c r="AT9" s="11" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="AU9" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV9" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW9" s="11" t="s">
         <v>74</v>
@@ -3347,7 +3927,7 @@
       </c>
       <c r="AY9" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X7RRBABA95</v>
+        <v>X1RSBABA8</v>
       </c>
       <c r="AZ9" s="24" t="s">
         <v>108</v>
@@ -3416,7 +3996,7 @@
         <v>119</v>
       </c>
       <c r="BV9" s="31">
-        <v>85328</v>
+        <v>33546</v>
       </c>
       <c r="BW9" s="24">
         <v>44562</v>
@@ -3430,10 +4010,14 @@
     </row>
     <row r="10" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
+        <v>191</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D10" s="10" t="s">
         <v>73</v>
       </c>
@@ -3443,10 +4027,14 @@
       <c r="F10" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G10" s="13"/>
-      <c r="H10" s="14"/>
+      <c r="G10" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>194</v>
+      </c>
       <c r="I10" s="15" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>79</v>
@@ -3456,7 +4044,7 @@
       </c>
       <c r="L10" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M10" s="11" t="s">
         <v>74</v>
@@ -3487,7 +4075,7 @@
       </c>
       <c r="V10" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W10" s="16" t="s">
         <v>87</v>
@@ -3521,7 +4109,7 @@
       </c>
       <c r="AG10" s="23">
         <f>V10+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH10" s="16" t="s">
         <v>150</v>
@@ -3534,34 +4122,34 @@
       </c>
       <c r="AK10" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL10" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM10" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN10" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO10" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP10" s="16" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="AQ10" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR10" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AS10" s="16" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AT10" s="11" t="s">
         <v>105</v>
@@ -3571,7 +4159,7 @@
       </c>
       <c r="AV10" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW10" s="11" t="s">
         <v>74</v>
@@ -3581,7 +4169,7 @@
       </c>
       <c r="AY10" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X1RRBABA83</v>
+        <v>X4RSBABA81</v>
       </c>
       <c r="AZ10" s="24" t="s">
         <v>108</v>
@@ -3650,7 +4238,7 @@
         <v>119</v>
       </c>
       <c r="BV10" s="31">
-        <v>85479</v>
+        <v>68030</v>
       </c>
       <c r="BW10" s="24">
         <v>44562</v>
@@ -3664,9 +4252,14 @@
     </row>
     <row r="11" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="C11" s="9"/>
+        <v>197</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D11" s="10" t="s">
         <v>73</v>
       </c>
@@ -3676,10 +4269,14 @@
       <c r="F11" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G11" s="13"/>
-      <c r="H11" s="14"/>
+      <c r="G11" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>200</v>
+      </c>
       <c r="I11" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J11" s="16" t="s">
         <v>79</v>
@@ -3689,7 +4286,7 @@
       </c>
       <c r="L11" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M11" s="11" t="s">
         <v>74</v>
@@ -3720,7 +4317,7 @@
       </c>
       <c r="V11" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W11" s="16" t="s">
         <v>87</v>
@@ -3732,7 +4329,7 @@
         <v>147</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="AA11" s="12" t="s">
         <v>149</v>
@@ -3750,11 +4347,11 @@
         <v>94</v>
       </c>
       <c r="AF11" s="12" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="AG11" s="23">
         <f>V11+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH11" s="16" t="s">
         <v>150</v>
@@ -3767,25 +4364,25 @@
       </c>
       <c r="AK11" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL11" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM11" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN11" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO11" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP11" s="16" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="AQ11" s="16" t="s">
         <v>102</v>
@@ -3797,14 +4394,14 @@
         <v>104</v>
       </c>
       <c r="AT11" s="11" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="AU11" s="11" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="AV11" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW11" s="11" t="s">
         <v>74</v>
@@ -3814,7 +4411,7 @@
       </c>
       <c r="AY11" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X4RRBABA33</v>
+        <v>X6RSBABA84</v>
       </c>
       <c r="AZ11" s="24" t="s">
         <v>108</v>
@@ -3883,7 +4480,7 @@
         <v>119</v>
       </c>
       <c r="BV11" s="31">
-        <v>57433</v>
+        <v>54648</v>
       </c>
       <c r="BW11" s="24">
         <v>44562</v>
@@ -3897,10 +4494,14 @@
     </row>
     <row r="12" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
+        <v>205</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D12" s="10" t="s">
         <v>73</v>
       </c>
@@ -3910,10 +4511,14 @@
       <c r="F12" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G12" s="13"/>
-      <c r="H12" s="14"/>
+      <c r="G12" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>208</v>
+      </c>
       <c r="I12" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>79</v>
@@ -3923,7 +4528,7 @@
       </c>
       <c r="L12" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M12" s="11" t="s">
         <v>74</v>
@@ -3954,7 +4559,7 @@
       </c>
       <c r="V12" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W12" s="16" t="s">
         <v>87</v>
@@ -3966,7 +4571,7 @@
         <v>89</v>
       </c>
       <c r="Z12" s="12" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="AA12" s="12" t="s">
         <v>91</v>
@@ -4000,15 +4605,15 @@
       </c>
       <c r="AK12" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL12" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM12" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN12" s="17">
         <f t="shared" si="5"/>
@@ -4018,7 +4623,7 @@
         <v>100</v>
       </c>
       <c r="AP12" s="16" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AQ12" s="16" t="s">
         <v>102</v>
@@ -4030,14 +4635,14 @@
         <v>104</v>
       </c>
       <c r="AT12" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AU12" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV12" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW12" s="11" t="s">
         <v>74</v>
@@ -4047,7 +4652,7 @@
       </c>
       <c r="AY12" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X9RRBABA61</v>
+        <v>X5RSBABA80</v>
       </c>
       <c r="AZ12" s="24" t="s">
         <v>108</v>
@@ -4116,7 +4721,7 @@
         <v>119</v>
       </c>
       <c r="BV12" s="31">
-        <v>36334</v>
+        <v>29230</v>
       </c>
       <c r="BW12" s="24">
         <v>44562</v>
@@ -4130,10 +4735,14 @@
     </row>
     <row r="13" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B13" s="35"/>
-      <c r="C13" s="9"/>
+        <v>210</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>211</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D13" s="10" t="s">
         <v>73</v>
       </c>
@@ -4143,10 +4752,14 @@
       <c r="F13" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="14"/>
+      <c r="G13" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>213</v>
+      </c>
       <c r="I13" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>79</v>
@@ -4156,7 +4769,7 @@
       </c>
       <c r="L13" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M13" s="11" t="s">
         <v>74</v>
@@ -4187,7 +4800,7 @@
       </c>
       <c r="V13" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W13" s="16" t="s">
         <v>87</v>
@@ -4196,10 +4809,10 @@
         <v>88</v>
       </c>
       <c r="Y13" s="12" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
       <c r="Z13" s="12" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
       <c r="AA13" s="12" t="s">
         <v>149</v>
@@ -4217,61 +4830,61 @@
         <v>94</v>
       </c>
       <c r="AF13" s="12" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="AG13" s="23">
         <f>V13+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH13" s="16" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
       <c r="AI13" s="16" t="s">
         <v>98</v>
       </c>
       <c r="AJ13" s="16" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="AK13" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL13" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM13" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN13" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO13" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP13" s="36" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="AQ13" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR13" s="16" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
       <c r="AS13" s="16" t="s">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="AT13" s="11" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="AU13" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV13" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW13" s="11" t="s">
         <v>74</v>
@@ -4281,7 +4894,7 @@
       </c>
       <c r="AY13" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X8RRBABA5</v>
+        <v>X7RSBABA34</v>
       </c>
       <c r="AZ13" s="24" t="s">
         <v>108</v>
@@ -4350,7 +4963,7 @@
         <v>119</v>
       </c>
       <c r="BV13" s="31">
-        <v>88076</v>
+        <v>51059</v>
       </c>
       <c r="BW13" s="24">
         <v>44562</v>
@@ -4364,9 +4977,14 @@
     </row>
     <row r="14" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C14" s="9"/>
+        <v>223</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D14" s="10" t="s">
         <v>73</v>
       </c>
@@ -4376,10 +4994,14 @@
       <c r="F14" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="13"/>
-      <c r="H14" s="14"/>
+      <c r="G14" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>226</v>
+      </c>
       <c r="I14" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>79</v>
@@ -4389,7 +5011,7 @@
       </c>
       <c r="L14" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M14" s="11" t="s">
         <v>74</v>
@@ -4420,7 +5042,7 @@
       </c>
       <c r="V14" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W14" s="16" t="s">
         <v>87</v>
@@ -4432,7 +5054,7 @@
         <v>89</v>
       </c>
       <c r="Z14" s="12" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="AA14" s="12" t="s">
         <v>91</v>
@@ -4466,15 +5088,15 @@
       </c>
       <c r="AK14" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL14" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM14" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN14" s="17">
         <f t="shared" si="5"/>
@@ -4484,26 +5106,26 @@
         <v>100</v>
       </c>
       <c r="AP14" s="16" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
       <c r="AQ14" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR14" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AS14" s="16" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="AT14" s="11" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="AU14" s="11" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="AV14" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW14" s="11" t="s">
         <v>74</v>
@@ -4513,7 +5135,7 @@
       </c>
       <c r="AY14" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X1RRBABA16</v>
+        <v>X7RSBABA63</v>
       </c>
       <c r="AZ14" s="24" t="s">
         <v>108</v>
@@ -4582,7 +5204,7 @@
         <v>119</v>
       </c>
       <c r="BV14" s="31">
-        <v>60463</v>
+        <v>37186</v>
       </c>
       <c r="BW14" s="24">
         <v>44562</v>
@@ -4596,10 +5218,14 @@
     </row>
     <row r="15" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="B15" s="35"/>
-      <c r="C15" s="9"/>
+        <v>232</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>233</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D15" s="10" t="s">
         <v>73</v>
       </c>
@@ -4609,10 +5235,14 @@
       <c r="F15" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="14"/>
+      <c r="G15" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>235</v>
+      </c>
       <c r="I15" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>79</v>
@@ -4622,7 +5252,7 @@
       </c>
       <c r="L15" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M15" s="11" t="s">
         <v>74</v>
@@ -4653,7 +5283,7 @@
       </c>
       <c r="V15" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W15" s="16" t="s">
         <v>87</v>
@@ -4665,7 +5295,7 @@
         <v>147</v>
       </c>
       <c r="Z15" s="12" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
       <c r="AA15" s="12" t="s">
         <v>149</v>
@@ -4687,7 +5317,7 @@
       </c>
       <c r="AG15" s="23">
         <f>V15+365</f>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AH15" s="16" t="s">
         <v>150</v>
@@ -4700,34 +5330,34 @@
       </c>
       <c r="AK15" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL15" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM15" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN15" s="17">
         <f t="shared" si="5"/>
-        <v>46088</v>
+        <v>46089</v>
       </c>
       <c r="AO15" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP15" s="16" t="s">
-        <v>212</v>
+        <v>236</v>
       </c>
       <c r="AQ15" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR15" s="16" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
       <c r="AS15" s="16" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AT15" s="11" t="s">
         <v>96</v>
@@ -4737,7 +5367,7 @@
       </c>
       <c r="AV15" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW15" s="11" t="s">
         <v>74</v>
@@ -4747,7 +5377,7 @@
       </c>
       <c r="AY15" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X2RRBABA88</v>
+        <v>X2RSBABA17</v>
       </c>
       <c r="AZ15" s="24" t="s">
         <v>108</v>
@@ -4816,7 +5446,7 @@
         <v>119</v>
       </c>
       <c r="BV15" s="31">
-        <v>70690</v>
+        <v>99531</v>
       </c>
       <c r="BW15" s="24">
         <v>44562</v>
@@ -4830,9 +5460,14 @@
     </row>
     <row r="16" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C16" s="9"/>
+        <v>237</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="D16" s="10" t="s">
         <v>73</v>
       </c>
@@ -4842,10 +5477,14 @@
       <c r="F16" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="14"/>
+      <c r="G16" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>240</v>
+      </c>
       <c r="I16" s="15" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>79</v>
@@ -4855,7 +5494,7 @@
       </c>
       <c r="L16" s="17">
         <f t="shared" si="0"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="M16" s="11" t="s">
         <v>74</v>
@@ -4886,7 +5525,7 @@
       </c>
       <c r="V16" s="17">
         <f t="shared" si="1"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="W16" s="16" t="s">
         <v>87</v>
@@ -4916,7 +5555,7 @@
         <v>94</v>
       </c>
       <c r="AF16" s="12" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="AG16" s="23" t="s">
         <v>96</v>
@@ -4932,15 +5571,15 @@
       </c>
       <c r="AK16" s="24">
         <f t="shared" si="2"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AL16" s="24">
         <f t="shared" si="3"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AM16" s="24">
         <f t="shared" si="4"/>
-        <v>45723</v>
+        <v>45724</v>
       </c>
       <c r="AN16" s="17">
         <f t="shared" si="5"/>
@@ -4950,16 +5589,16 @@
         <v>100</v>
       </c>
       <c r="AP16" s="16" t="s">
-        <v>214</v>
+        <v>241</v>
       </c>
       <c r="AQ16" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR16" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AS16" s="16" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AT16" s="11" t="s">
         <v>105</v>
@@ -4969,7 +5608,7 @@
       </c>
       <c r="AV16" s="24">
         <f t="shared" si="6"/>
-        <v>45774</v>
+        <v>45775</v>
       </c>
       <c r="AW16" s="11" t="s">
         <v>74</v>
@@ -4979,7 +5618,7 @@
       </c>
       <c r="AY16" s="26" t="str">
         <f t="shared" si="7"/>
-        <v>X5RRBABA2</v>
+        <v>X6RSBABA53</v>
       </c>
       <c r="AZ16" s="24" t="s">
         <v>108</v>
@@ -5048,7 +5687,7 @@
         <v>119</v>
       </c>
       <c r="BV16" s="31">
-        <v>44210</v>
+        <v>56573</v>
       </c>
       <c r="BW16" s="24">
         <v>44562</v>
@@ -5060,432 +5699,608 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" ht="15.65" customHeight="1" spans="38:38" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.65" customHeight="1" spans="2:38" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C17" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AL17" s="24"/>
     </row>
-    <row r="28" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G18" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C21" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G22" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C23" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G24" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G26" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="27" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G27" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="28" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B28" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C28" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX28" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY28" s="37">
+        <v>259</v>
+      </c>
+      <c r="AY28" s="38">
         <f t="array" ref="AY28:AY47">_xlfn.RANDARRAY(20,1,1,9,TRUE)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AZ28" s="26" t="s">
-        <v>216</v>
-      </c>
-      <c r="BA28" s="37">
+        <v>260</v>
+      </c>
+      <c r="BA28" s="38">
         <f t="array" ref="BA28:BA47">_xlfn.RANDARRAY(20,1,1,99,TRUE)</f>
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="BB28" s="1" t="str">
         <f>AX28&amp;AY28&amp;AZ28&amp;BA28</f>
-        <v>X6RRBABA21</v>
+        <v>X1RSBABA18</v>
       </c>
     </row>
-    <row r="29" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="29" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G29" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>262</v>
+      </c>
       <c r="AX29" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY29" s="37">
-        <v>2</v>
+        <v>259</v>
+      </c>
+      <c r="AY29" s="38">
+        <v>5</v>
       </c>
       <c r="AZ29" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA29" s="2">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="BB29" s="1" t="str">
         <f t="shared" ref="BB29:BB53" si="8">AX29&amp;AY29&amp;AZ29&amp;BA29</f>
-        <v>X2RRBABA34</v>
+        <v>X5RSBABA47</v>
       </c>
     </row>
-    <row r="30" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="30" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B30" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C30" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX30" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY30" s="37">
-        <v>2</v>
+        <v>259</v>
+      </c>
+      <c r="AY30" s="38">
+        <v>3</v>
       </c>
       <c r="AZ30" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA30" s="2">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="BB30" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X2RRBABA36</v>
+        <v>X3RSBABA79</v>
       </c>
     </row>
-    <row r="31" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="31" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B31" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C31" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX31" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY31" s="37">
-        <v>3</v>
+        <v>259</v>
+      </c>
+      <c r="AY31" s="38">
+        <v>7</v>
       </c>
       <c r="AZ31" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA31" s="2">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="BB31" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X3RRBABA41</v>
+        <v>X7RSBABA2</v>
       </c>
     </row>
-    <row r="32" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="32" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B32" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C32" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX32" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY32" s="37">
-        <v>5</v>
+        <v>259</v>
+      </c>
+      <c r="AY32" s="38">
+        <v>3</v>
       </c>
       <c r="AZ32" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA32" s="2">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="BB32" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X5RRBABA26</v>
+        <v>X3RSBABA91</v>
       </c>
     </row>
-    <row r="33" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="33" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B33" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C33" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX33" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY33" s="37">
-        <v>4</v>
+        <v>259</v>
+      </c>
+      <c r="AY33" s="38">
+        <v>8</v>
       </c>
       <c r="AZ33" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA33" s="2">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="BB33" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X4RRBABA70</v>
+        <v>X8RSBABA76</v>
       </c>
     </row>
-    <row r="34" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="34" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G34" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>268</v>
+      </c>
       <c r="AX34" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY34" s="37">
-        <v>7</v>
+        <v>259</v>
+      </c>
+      <c r="AY34" s="38">
+        <v>1</v>
       </c>
       <c r="AZ34" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA34" s="2">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="BB34" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X7RRBABA41</v>
+        <v>X1RSBABA81</v>
       </c>
     </row>
-    <row r="35" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="35" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G35" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>270</v>
+      </c>
       <c r="AX35" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY35" s="37">
-        <v>7</v>
+        <v>259</v>
+      </c>
+      <c r="AY35" s="38">
+        <v>1</v>
       </c>
       <c r="AZ35" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA35" s="2">
-        <v>95</v>
+        <v>8</v>
       </c>
       <c r="BB35" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X7RRBABA95</v>
+        <v>X1RSBABA8</v>
       </c>
     </row>
-    <row r="36" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="36" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G36" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>272</v>
+      </c>
       <c r="AX36" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY36" s="37">
-        <v>1</v>
+        <v>259</v>
+      </c>
+      <c r="AY36" s="38">
+        <v>4</v>
       </c>
       <c r="AZ36" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA36" s="2">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="BB36" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X1RRBABA83</v>
+        <v>X4RSBABA81</v>
       </c>
     </row>
-    <row r="37" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="37" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G37" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>274</v>
+      </c>
       <c r="AX37" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY37" s="37">
-        <v>4</v>
+        <v>259</v>
+      </c>
+      <c r="AY37" s="38">
+        <v>6</v>
       </c>
       <c r="AZ37" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA37" s="2">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="BB37" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X4RRBABA33</v>
+        <v>X6RSBABA84</v>
       </c>
     </row>
-    <row r="38" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="38" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B38" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C38" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX38" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY38" s="37">
-        <v>9</v>
+        <v>259</v>
+      </c>
+      <c r="AY38" s="38">
+        <v>5</v>
       </c>
       <c r="AZ38" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA38" s="2">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="BB38" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X9RRBABA61</v>
+        <v>X5RSBABA80</v>
       </c>
     </row>
-    <row r="39" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="39" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G39" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>277</v>
+      </c>
       <c r="AX39" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY39" s="37">
-        <v>8</v>
+        <v>259</v>
+      </c>
+      <c r="AY39" s="38">
+        <v>7</v>
       </c>
       <c r="AZ39" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA39" s="2">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="BB39" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X8RRBABA5</v>
+        <v>X7RSBABA34</v>
       </c>
     </row>
-    <row r="40" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="40" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G40" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>279</v>
+      </c>
       <c r="AX40" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY40" s="37">
-        <v>1</v>
+        <v>259</v>
+      </c>
+      <c r="AY40" s="38">
+        <v>7</v>
       </c>
       <c r="AZ40" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA40" s="2">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="BB40" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X1RRBABA16</v>
+        <v>X7RSBABA63</v>
       </c>
     </row>
-    <row r="41" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="41" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
+      <c r="G41" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>281</v>
+      </c>
       <c r="AX41" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY41" s="37">
+        <v>259</v>
+      </c>
+      <c r="AY41" s="38">
         <v>2</v>
       </c>
       <c r="AZ41" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA41" s="2">
-        <v>88</v>
+        <v>17</v>
       </c>
       <c r="BB41" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X2RRBABA88</v>
+        <v>X2RSBABA17</v>
       </c>
     </row>
-    <row r="42" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
+    <row r="42" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
+      <c r="B42" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C42" s="37" t="s">
+        <v>137</v>
+      </c>
       <c r="AX42" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY42" s="37">
-        <v>5</v>
+        <v>259</v>
+      </c>
+      <c r="AY42" s="38">
+        <v>6</v>
       </c>
       <c r="AZ42" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA42" s="2">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="BB42" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X5RRBABA2</v>
+        <v>X6RSBABA53</v>
       </c>
     </row>
     <row r="43" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX43" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY43" s="37">
-        <v>3</v>
+        <v>259</v>
+      </c>
+      <c r="AY43" s="38">
+        <v>9</v>
       </c>
       <c r="AZ43" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA43" s="2">
-        <v>74</v>
+        <v>4</v>
       </c>
       <c r="BB43" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X3RRBABA74</v>
+        <v>X9RSBABA4</v>
       </c>
     </row>
     <row r="44" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX44" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY44" s="37">
-        <v>6</v>
+        <v>259</v>
+      </c>
+      <c r="AY44" s="38">
+        <v>2</v>
       </c>
       <c r="AZ44" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA44" s="2">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="BB44" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X6RRBABA37</v>
+        <v>X2RSBABA74</v>
       </c>
     </row>
     <row r="45" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX45" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY45" s="37">
-        <v>1</v>
+        <v>259</v>
+      </c>
+      <c r="AY45" s="38">
+        <v>7</v>
       </c>
       <c r="AZ45" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA45" s="2">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="BB45" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X1RRBABA52</v>
+        <v>X7RSBABA51</v>
       </c>
     </row>
     <row r="46" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX46" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY46" s="37">
-        <v>8</v>
+        <v>259</v>
+      </c>
+      <c r="AY46" s="38">
+        <v>1</v>
       </c>
       <c r="AZ46" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA46" s="2">
-        <v>18</v>
+        <v>59</v>
       </c>
       <c r="BB46" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X8RRBABA18</v>
+        <v>X1RSBABA59</v>
       </c>
     </row>
     <row r="47" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX47" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY47" s="37">
-        <v>3</v>
+        <v>259</v>
+      </c>
+      <c r="AY47" s="38">
+        <v>2</v>
       </c>
       <c r="AZ47" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BA47" s="2">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="BB47" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>X3RRBABA36</v>
+        <v>X2RSBABA16</v>
       </c>
     </row>
     <row r="48" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX48" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY48" s="37"/>
+        <v>259</v>
+      </c>
+      <c r="AY48" s="38"/>
       <c r="AZ48" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BB48" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>XRRBABA</v>
+        <v>XRSBABA</v>
       </c>
     </row>
     <row r="49" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX49" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY49" s="37"/>
+        <v>259</v>
+      </c>
+      <c r="AY49" s="38"/>
       <c r="AZ49" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BB49" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>XRRBABA</v>
+        <v>XRSBABA</v>
       </c>
     </row>
     <row r="50" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX50" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="AY50" s="37"/>
+        <v>259</v>
+      </c>
+      <c r="AY50" s="38"/>
       <c r="AZ50" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BB50" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>XRRBABA</v>
+        <v>XRSBABA</v>
       </c>
     </row>
     <row r="51" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX51" s="1" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="AZ51" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BB51" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>XRRBABA</v>
+        <v>XRSBABA</v>
       </c>
     </row>
     <row r="52" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX52" s="1" t="s">
-        <v>215</v>
+        <v>259</v>
       </c>
       <c r="AZ52" s="26" t="s">
-        <v>216</v>
+        <v>260</v>
       </c>
       <c r="BB52" s="1" t="str">
         <f t="shared" si="8"/>
-        <v>XRRBABA</v>
+        <v>XRSBABA</v>
       </c>
     </row>
     <row r="53" ht="15.65" customHeight="1" spans="54:54" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Latest code for Italy
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataFranceMK.xlsx
+++ b/Data/Hires/TestDataFranceMK.xlsx
@@ -1,30 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{164A78DA-73A9-45FE-8847-9D3673460A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -439,232 +424,235 @@
     <t>Test4</t>
   </si>
   <si>
+    <t>Renee</t>
+  </si>
+  <si>
+    <t>Lang</t>
+  </si>
+  <si>
+    <t>Auto 28725953</t>
+  </si>
+  <si>
+    <t>Department Manager</t>
+  </si>
+  <si>
+    <t>France Department Manager</t>
+  </si>
+  <si>
+    <t>Test5</t>
+  </si>
+  <si>
+    <t>Bailee</t>
+  </si>
+  <si>
+    <t>Kunze</t>
+  </si>
+  <si>
+    <t>Auto 34305455</t>
+  </si>
+  <si>
+    <t>Fixed Term (Fixed Term)</t>
+  </si>
+  <si>
+    <t>Senior Department Manager</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>CDD (Durée determinée)</t>
+  </si>
+  <si>
+    <t>Cadre</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>France Senior Department Manager</t>
+  </si>
+  <si>
+    <t>MrunB</t>
+  </si>
+  <si>
+    <t>FrunB</t>
+  </si>
+  <si>
+    <t>Test6</t>
+  </si>
+  <si>
+    <t>10698403</t>
+  </si>
+  <si>
+    <t>Korbin</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>Auto 94727550</t>
+  </si>
+  <si>
+    <t>Trainee Manager</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>France Trainee Manager</t>
+  </si>
+  <si>
+    <t>Test7</t>
+  </si>
+  <si>
+    <t>10698404</t>
+  </si>
+  <si>
+    <t>Krystal</t>
+  </si>
+  <si>
+    <t>Sipes</t>
+  </si>
+  <si>
+    <t>4 48 29 85 70</t>
+  </si>
+  <si>
+    <t>Auto 53957765</t>
+  </si>
+  <si>
+    <t>Assistant Manager</t>
+  </si>
+  <si>
+    <t>France Assistant Manager</t>
+  </si>
+  <si>
+    <t>Test8</t>
+  </si>
+  <si>
+    <t>10698405</t>
+  </si>
+  <si>
+    <t>Ocie</t>
+  </si>
+  <si>
+    <t>Macejkovic</t>
+  </si>
+  <si>
+    <t>5 48 29 85 70</t>
+  </si>
+  <si>
+    <t>P&amp;C Assistant (NLD/FRA/USA/ITA/PL/CZ ONLY)</t>
+  </si>
+  <si>
+    <t>250 Human Resources Retail</t>
+  </si>
+  <si>
+    <t>Employé</t>
+  </si>
+  <si>
+    <t>E3</t>
+  </si>
+  <si>
+    <t>France P&amp;C Assistant/P&amp;C Supervisor</t>
+  </si>
+  <si>
+    <t>Test9</t>
+  </si>
+  <si>
+    <t>221 Store Management (Rykil Wuhoga (9221018))</t>
+  </si>
+  <si>
+    <t>Crystel</t>
+  </si>
+  <si>
+    <t>Schinner</t>
+  </si>
+  <si>
+    <t>6 48 29 85 70</t>
+  </si>
+  <si>
+    <t>Auto 09112024 230837</t>
+  </si>
+  <si>
+    <t>P&amp;C Manager Stores</t>
+  </si>
+  <si>
+    <t>France P&amp;C Manager</t>
+  </si>
+  <si>
+    <t>Test10</t>
+  </si>
+  <si>
+    <t>10698406</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Krajcik</t>
+  </si>
+  <si>
+    <t>7 48 29 85 70</t>
+  </si>
+  <si>
+    <t>255 Stockroom</t>
+  </si>
+  <si>
+    <t>Test11</t>
+  </si>
+  <si>
+    <t>10698407</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Vandervort</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
+  </si>
+  <si>
+    <t>2 jours (France)</t>
+  </si>
+  <si>
+    <t>253 Supervisors</t>
+  </si>
+  <si>
+    <t>France Supervisor</t>
+  </si>
+  <si>
+    <t>Test12</t>
+  </si>
+  <si>
+    <t>10698408</t>
+  </si>
+  <si>
+    <t>Lester</t>
+  </si>
+  <si>
+    <t>Nicolas</t>
+  </si>
+  <si>
+    <t>P&amp;C Supervisor (NLD/FRA/USA/ITA/PL/CZ ONLY)</t>
+  </si>
+  <si>
+    <t>Test13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'Oceane Heaney' Employee:{undefined}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for locator('text=Propose Compensation Hire:  Oceane Heaney')[22m
+</t>
+  </si>
+  <si>
     <t>Failed</t>
   </si>
   <si>
-    <t>Renee</t>
-  </si>
-  <si>
-    <t>Lang</t>
-  </si>
-  <si>
-    <t>Auto 28725953</t>
-  </si>
-  <si>
-    <t>Department Manager</t>
-  </si>
-  <si>
-    <t>France Department Manager</t>
-  </si>
-  <si>
-    <t>Test5</t>
-  </si>
-  <si>
-    <t>Bailee</t>
-  </si>
-  <si>
-    <t>Kunze</t>
-  </si>
-  <si>
-    <t>Auto 34305455</t>
-  </si>
-  <si>
-    <t>Fixed Term (Fixed Term)</t>
-  </si>
-  <si>
-    <t>Senior Department Manager</t>
-  </si>
-  <si>
-    <t>Part time</t>
-  </si>
-  <si>
-    <t>CDD (Durée determinée)</t>
-  </si>
-  <si>
-    <t>Cadre</t>
-  </si>
-  <si>
-    <t>C2</t>
-  </si>
-  <si>
-    <t>France Senior Department Manager</t>
-  </si>
-  <si>
-    <t>MrunB</t>
-  </si>
-  <si>
-    <t>FrunB</t>
-  </si>
-  <si>
-    <t>Test6</t>
-  </si>
-  <si>
-    <t>10698403</t>
-  </si>
-  <si>
-    <t>Korbin</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>Auto 94727550</t>
-  </si>
-  <si>
-    <t>Trainee Manager</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>France Trainee Manager</t>
-  </si>
-  <si>
-    <t>Test7</t>
-  </si>
-  <si>
-    <t>10698404</t>
-  </si>
-  <si>
-    <t>Krystal</t>
-  </si>
-  <si>
-    <t>Sipes</t>
-  </si>
-  <si>
-    <t>4 48 29 85 70</t>
-  </si>
-  <si>
-    <t>Auto 53957765</t>
-  </si>
-  <si>
-    <t>Assistant Manager</t>
-  </si>
-  <si>
-    <t>France Assistant Manager</t>
-  </si>
-  <si>
-    <t>Test8</t>
-  </si>
-  <si>
-    <t>10698405</t>
-  </si>
-  <si>
-    <t>Ocie</t>
-  </si>
-  <si>
-    <t>Macejkovic</t>
-  </si>
-  <si>
-    <t>5 48 29 85 70</t>
-  </si>
-  <si>
-    <t>P&amp;C Assistant (NLD/FRA/USA/ITA/PL/CZ ONLY)</t>
-  </si>
-  <si>
-    <t>250 Human Resources Retail</t>
-  </si>
-  <si>
-    <t>Employé</t>
-  </si>
-  <si>
-    <t>E3</t>
-  </si>
-  <si>
-    <t>France P&amp;C Assistant/P&amp;C Supervisor</t>
-  </si>
-  <si>
-    <t>Test9</t>
-  </si>
-  <si>
-    <t>221 Store Management (Rykil Wuhoga (9221018))</t>
-  </si>
-  <si>
-    <t>Crystel</t>
-  </si>
-  <si>
-    <t>Schinner</t>
-  </si>
-  <si>
-    <t>6 48 29 85 70</t>
-  </si>
-  <si>
-    <t>Auto 09112024 230837</t>
-  </si>
-  <si>
-    <t>P&amp;C Manager Stores</t>
-  </si>
-  <si>
-    <t>France P&amp;C Manager</t>
-  </si>
-  <si>
-    <t>Test10</t>
-  </si>
-  <si>
-    <t>10698406</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>Krajcik</t>
-  </si>
-  <si>
-    <t>7 48 29 85 70</t>
-  </si>
-  <si>
-    <t>255 Stockroom</t>
-  </si>
-  <si>
-    <t>Test11</t>
-  </si>
-  <si>
-    <t>10698407</t>
-  </si>
-  <si>
-    <t>Santiago</t>
-  </si>
-  <si>
-    <t>Vandervort</t>
-  </si>
-  <si>
-    <t>Supervisor</t>
-  </si>
-  <si>
-    <t>2 jours (France)</t>
-  </si>
-  <si>
-    <t>253 Supervisors</t>
-  </si>
-  <si>
-    <t>France Supervisor</t>
-  </si>
-  <si>
-    <t>Test12</t>
-  </si>
-  <si>
-    <t>10698408</t>
-  </si>
-  <si>
-    <t>Lester</t>
-  </si>
-  <si>
-    <t>Nicolas</t>
-  </si>
-  <si>
-    <t>P&amp;C Supervisor (NLD/FRA/USA/ITA/PL/CZ ONLY)</t>
-  </si>
-  <si>
-    <t>Test13</t>
-  </si>
-  <si>
-    <t>10698409</t>
-  </si>
-  <si>
-    <t>Dedrick</t>
-  </si>
-  <si>
-    <t>Turcotte</t>
+    <t>Oceane</t>
+  </si>
+  <si>
+    <t>Heaney</t>
   </si>
   <si>
     <t>Contrat apprentissage</t>
@@ -697,13 +685,13 @@
     <t>Test14</t>
   </si>
   <si>
-    <t>10698410</t>
-  </si>
-  <si>
-    <t>Meghan</t>
-  </si>
-  <si>
-    <t>Thiel</t>
+    <t>10698579</t>
+  </si>
+  <si>
+    <t>Lina</t>
+  </si>
+  <si>
+    <t>Grant</t>
   </si>
   <si>
     <t>Visuel Merchandiser</t>
@@ -724,13 +712,15 @@
     <t>Test15</t>
   </si>
   <si>
-    <t>10698411</t>
-  </si>
-  <si>
-    <t>Sadye</t>
-  </si>
-  <si>
-    <t>Durgan</t>
+    <t xml:space="preserve">Test failed for 'David Ziemann' Employee:{10698581}Error: [2mexpect([22m[31mreceived[39m[2m).[22mtoEqual[2m([22m[32mexpected[39m[2m) // deep equality[22m
+Expected: [32m"FR Monthly"[39m
+Received: [31m"Please select a French Pay Group"[39m</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Ziemann</t>
   </si>
   <si>
     <t>08 Ladieswear</t>
@@ -877,68 +867,68 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FFFF0000"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -947,24 +937,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -972,11 +962,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -995,60 +980,38 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1150,9 +1113,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1436,9 +1396,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BY53"/>
-  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="10.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.36328125" style="1" customWidth="1"/>
@@ -1518,7 +1478,7 @@
     <col min="77" max="77" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:77" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.5" customHeight="1" spans="1:77" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1751,7 +1711,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>70</v>
       </c>
@@ -1786,7 +1746,7 @@
         <v>80</v>
       </c>
       <c r="L2" s="17">
-        <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="L2:L16" si="0">TODAY()-31</f>
         <v>45725</v>
       </c>
       <c r="M2" s="11" t="s">
@@ -1817,7 +1777,7 @@
         <v>80</v>
       </c>
       <c r="V2" s="17">
-        <f t="shared" ref="V2:V16" ca="1" si="1">L2</f>
+        <f t="shared" ref="V2:V16" si="1">L2</f>
         <v>45725</v>
       </c>
       <c r="W2" s="16" t="s">
@@ -1863,20 +1823,20 @@
         <v>99</v>
       </c>
       <c r="AK2" s="24">
-        <f t="shared" ref="AK2:AK16" ca="1" si="2">V2</f>
+        <f t="shared" ref="AK2:AK16" si="2">V2</f>
         <v>45725</v>
       </c>
       <c r="AL2" s="24">
-        <f t="shared" ref="AL2:AL16" ca="1" si="3">V2</f>
+        <f t="shared" ref="AL2:AL16" si="3">V2</f>
         <v>45725</v>
       </c>
       <c r="AM2" s="24">
-        <f t="shared" ref="AM2:AM16" ca="1" si="4">V2</f>
-        <v>45725</v>
-      </c>
-      <c r="AN2" s="17" t="str">
+        <f t="shared" ref="AM2:AM16" si="4">V2</f>
+        <v>45725</v>
+      </c>
+      <c r="AN2" s="17">
         <f t="shared" ref="AN2:AN16" si="5">AG2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO2" s="16" t="s">
         <v>100</v>
@@ -1900,7 +1860,7 @@
         <v>106</v>
       </c>
       <c r="AV2" s="24">
-        <f t="shared" ref="AV2:AV16" ca="1" si="6">TODAY()+20</f>
+        <f t="shared" ref="AV2:AV16" si="6">TODAY()+20</f>
         <v>45776</v>
       </c>
       <c r="AW2" s="11" t="s">
@@ -1910,7 +1870,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="26" t="str">
-        <f ca="1">BB28</f>
+        <f>BB28</f>
         <v>X7RSBABA74</v>
       </c>
       <c r="AZ2" s="24" t="s">
@@ -1980,7 +1940,7 @@
         <v>119</v>
       </c>
       <c r="BV2" s="31">
-        <f t="array" aca="1" ref="BV2:BV16" ca="1">_xlfn.RANDARRAY(15,1,12345,99999,TRUE)</f>
+        <f t="array" ref="BV2:BV16">_xlfn.RANDARRAY(15,1,12345,99999,TRUE)</f>
         <v>49975</v>
       </c>
       <c r="BW2" s="24">
@@ -1993,7 +1953,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>121</v>
       </c>
@@ -2028,7 +1988,7 @@
         <v>80</v>
       </c>
       <c r="L3" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M3" s="11" t="s">
@@ -2059,7 +2019,7 @@
         <v>80</v>
       </c>
       <c r="V3" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W3" s="16" t="s">
@@ -2105,20 +2065,20 @@
         <v>99</v>
       </c>
       <c r="AK3" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL3" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM3" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN3" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN3" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO3" s="16" t="s">
         <v>129</v>
@@ -2142,7 +2102,7 @@
         <v>96</v>
       </c>
       <c r="AV3" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW3" s="11" t="s">
@@ -2152,7 +2112,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="26" t="str">
-        <f t="shared" ref="AY3:AY16" ca="1" si="7">BB29</f>
+        <f t="shared" ref="AY3:AY16" si="7">BB29</f>
         <v>X7RSBABA15</v>
       </c>
       <c r="AZ3" s="24" t="s">
@@ -2222,7 +2182,6 @@
         <v>119</v>
       </c>
       <c r="BV3" s="31">
-        <f ca="1"/>
         <v>73179</v>
       </c>
       <c r="BW3" s="24">
@@ -2235,7 +2194,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>135</v>
       </c>
@@ -2250,10 +2209,10 @@
         <v>75</v>
       </c>
       <c r="G4" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>137</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>138</v>
       </c>
       <c r="I4" s="15" t="s">
         <v>78</v>
@@ -2265,7 +2224,7 @@
         <v>80</v>
       </c>
       <c r="L4" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M4" s="11" t="s">
@@ -2296,20 +2255,20 @@
         <v>80</v>
       </c>
       <c r="V4" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W4" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X4" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="Y4" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z4" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AA4" s="12" t="s">
         <v>91</v>
@@ -2342,20 +2301,20 @@
         <v>99</v>
       </c>
       <c r="AK4" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL4" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM4" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN4" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN4" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO4" s="16" t="s">
         <v>129</v>
@@ -2373,13 +2332,13 @@
         <v>104</v>
       </c>
       <c r="AT4" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AU4" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV4" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW4" s="11" t="s">
@@ -2389,7 +2348,7 @@
         <v>107</v>
       </c>
       <c r="AY4" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X8RSBABA3</v>
       </c>
       <c r="AZ4" s="24" t="s">
@@ -2459,7 +2418,6 @@
         <v>119</v>
       </c>
       <c r="BV4" s="31">
-        <f ca="1"/>
         <v>17263</v>
       </c>
       <c r="BW4" s="24">
@@ -2472,9 +2430,9 @@
         <v>120</v>
       </c>
     </row>
-    <row r="5" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="10" t="s">
@@ -2487,10 +2445,10 @@
         <v>75</v>
       </c>
       <c r="G5" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="I5" s="15" t="s">
         <v>78</v>
@@ -2502,7 +2460,7 @@
         <v>80</v>
       </c>
       <c r="L5" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M5" s="11" t="s">
@@ -2533,23 +2491,23 @@
         <v>80</v>
       </c>
       <c r="V5" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W5" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X5" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="Y5" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="Y5" s="12" t="s">
+      <c r="Z5" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="Z5" s="12" t="s">
+      <c r="AA5" s="12" t="s">
         <v>147</v>
-      </c>
-      <c r="AA5" s="12" t="s">
-        <v>148</v>
       </c>
       <c r="AB5" s="20" t="s">
         <v>92</v>
@@ -2567,11 +2525,11 @@
         <v>95</v>
       </c>
       <c r="AG5" s="23">
-        <f ca="1">V5+365</f>
+        <f>V5+365</f>
         <v>46090</v>
       </c>
       <c r="AH5" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AI5" s="16" t="s">
         <v>98</v>
@@ -2580,19 +2538,19 @@
         <v>99</v>
       </c>
       <c r="AK5" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL5" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM5" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN5" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO5" s="16" t="s">
@@ -2605,19 +2563,19 @@
         <v>102</v>
       </c>
       <c r="AR5" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="AS5" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="AS5" s="16" t="s">
+      <c r="AT5" s="32" t="s">
         <v>151</v>
-      </c>
-      <c r="AT5" s="32" t="s">
-        <v>152</v>
       </c>
       <c r="AU5" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV5" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW5" s="11" t="s">
@@ -2627,7 +2585,7 @@
         <v>107</v>
       </c>
       <c r="AY5" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X9RSBABA65</v>
       </c>
       <c r="AZ5" s="24" t="s">
@@ -2685,10 +2643,10 @@
         <v>74</v>
       </c>
       <c r="BR5" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS5" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS5" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT5" s="11" t="s">
         <v>74</v>
@@ -2697,7 +2655,6 @@
         <v>119</v>
       </c>
       <c r="BV5" s="31">
-        <f ca="1"/>
         <v>72470</v>
       </c>
       <c r="BW5" s="24">
@@ -2710,12 +2667,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>156</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>72</v>
@@ -2730,10 +2687,10 @@
         <v>75</v>
       </c>
       <c r="G6" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="H6" s="14" t="s">
         <v>157</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>158</v>
       </c>
       <c r="I6" s="15" t="s">
         <v>78</v>
@@ -2745,7 +2702,7 @@
         <v>80</v>
       </c>
       <c r="L6" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M6" s="11" t="s">
@@ -2776,20 +2733,20 @@
         <v>80</v>
       </c>
       <c r="V6" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W6" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X6" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="Y6" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z6" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AA6" s="12" t="s">
         <v>91</v>
@@ -2822,20 +2779,20 @@
         <v>99</v>
       </c>
       <c r="AK6" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL6" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM6" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN6" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN6" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO6" s="16" t="s">
         <v>129</v>
@@ -2847,19 +2804,19 @@
         <v>102</v>
       </c>
       <c r="AR6" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AS6" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="AT6" s="11" t="s">
         <v>161</v>
-      </c>
-      <c r="AT6" s="11" t="s">
-        <v>162</v>
       </c>
       <c r="AU6" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV6" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW6" s="11" t="s">
@@ -2869,7 +2826,7 @@
         <v>107</v>
       </c>
       <c r="AY6" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X8RSBABA96</v>
       </c>
       <c r="AZ6" s="24" t="s">
@@ -2927,10 +2884,10 @@
         <v>74</v>
       </c>
       <c r="BR6" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS6" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS6" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT6" s="11" t="s">
         <v>74</v>
@@ -2939,7 +2896,6 @@
         <v>119</v>
       </c>
       <c r="BV6" s="31">
-        <f ca="1"/>
         <v>70223</v>
       </c>
       <c r="BW6" s="24">
@@ -2952,12 +2908,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:77" s="33" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B7" s="34" t="s">
         <v>163</v>
-      </c>
-      <c r="B7" s="34" t="s">
-        <v>164</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>72</v>
@@ -2972,13 +2928,13 @@
         <v>75</v>
       </c>
       <c r="G7" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="H7" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="I7" s="15" t="s">
         <v>166</v>
-      </c>
-      <c r="I7" s="15" t="s">
-        <v>167</v>
       </c>
       <c r="J7" s="16" t="s">
         <v>79</v>
@@ -2987,7 +2943,7 @@
         <v>80</v>
       </c>
       <c r="L7" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M7" s="11" t="s">
@@ -3018,20 +2974,20 @@
         <v>80</v>
       </c>
       <c r="V7" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W7" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X7" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="Y7" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z7" s="12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="AA7" s="12" t="s">
         <v>91</v>
@@ -3064,20 +3020,20 @@
         <v>99</v>
       </c>
       <c r="AK7" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL7" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM7" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN7" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN7" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO7" s="16" t="s">
         <v>129</v>
@@ -3089,19 +3045,19 @@
         <v>102</v>
       </c>
       <c r="AR7" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="AS7" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="AS7" s="16" t="s">
-        <v>151</v>
-      </c>
       <c r="AT7" s="32" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AU7" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV7" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW7" s="11" t="s">
@@ -3111,7 +3067,7 @@
         <v>107</v>
       </c>
       <c r="AY7" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X1RSBABA20</v>
       </c>
       <c r="AZ7" s="24" t="s">
@@ -3169,10 +3125,10 @@
         <v>74</v>
       </c>
       <c r="BR7" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS7" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS7" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT7" s="11" t="s">
         <v>74</v>
@@ -3181,7 +3137,6 @@
         <v>119</v>
       </c>
       <c r="BV7" s="31">
-        <f ca="1"/>
         <v>97454</v>
       </c>
       <c r="BW7" s="24">
@@ -3194,12 +3149,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="1:77" s="33" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>171</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>172</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>72</v>
@@ -3214,13 +3169,13 @@
         <v>75</v>
       </c>
       <c r="G8" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="H8" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="I8" s="15" t="s">
         <v>174</v>
-      </c>
-      <c r="I8" s="15" t="s">
-        <v>175</v>
       </c>
       <c r="J8" s="16" t="s">
         <v>79</v>
@@ -3229,7 +3184,7 @@
         <v>80</v>
       </c>
       <c r="L8" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M8" s="11" t="s">
@@ -3260,7 +3215,7 @@
         <v>80</v>
       </c>
       <c r="V8" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W8" s="16" t="s">
@@ -3270,13 +3225,13 @@
         <v>88</v>
       </c>
       <c r="Y8" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Z8" s="12" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AA8" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB8" s="20" t="s">
         <v>92</v>
@@ -3294,11 +3249,11 @@
         <v>95</v>
       </c>
       <c r="AG8" s="23">
-        <f ca="1">V8+365</f>
+        <f>V8+365</f>
         <v>46090</v>
       </c>
       <c r="AH8" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AI8" s="16" t="s">
         <v>98</v>
@@ -3307,44 +3262,44 @@
         <v>99</v>
       </c>
       <c r="AK8" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL8" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM8" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN8" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO8" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP8" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AQ8" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR8" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="AS8" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="AS8" s="16" t="s">
+      <c r="AT8" s="11" t="s">
         <v>179</v>
-      </c>
-      <c r="AT8" s="11" t="s">
-        <v>180</v>
       </c>
       <c r="AU8" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV8" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW8" s="11" t="s">
@@ -3354,7 +3309,7 @@
         <v>107</v>
       </c>
       <c r="AY8" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X2RSBABA59</v>
       </c>
       <c r="AZ8" s="24" t="s">
@@ -3412,10 +3367,10 @@
         <v>74</v>
       </c>
       <c r="BR8" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS8" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS8" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT8" s="11" t="s">
         <v>74</v>
@@ -3424,7 +3379,6 @@
         <v>119</v>
       </c>
       <c r="BV8" s="31">
-        <f ca="1"/>
         <v>94134</v>
       </c>
       <c r="BW8" s="24">
@@ -3437,13 +3391,13 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C9" s="9"/>
       <c r="D9" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>74</v>
@@ -3452,13 +3406,13 @@
         <v>75</v>
       </c>
       <c r="G9" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="H9" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="I9" s="15" t="s">
         <v>184</v>
-      </c>
-      <c r="I9" s="15" t="s">
-        <v>185</v>
       </c>
       <c r="J9" s="16" t="s">
         <v>79</v>
@@ -3467,7 +3421,7 @@
         <v>80</v>
       </c>
       <c r="L9" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M9" s="11" t="s">
@@ -3498,20 +3452,20 @@
         <v>80</v>
       </c>
       <c r="V9" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W9" s="16" t="s">
         <v>87</v>
       </c>
       <c r="X9" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Y9" s="12" t="s">
         <v>89</v>
       </c>
       <c r="Z9" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AA9" s="12" t="s">
         <v>91</v>
@@ -3544,20 +3498,20 @@
         <v>99</v>
       </c>
       <c r="AK9" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL9" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM9" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN9" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN9" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO9" s="16" t="s">
         <v>129</v>
@@ -3569,19 +3523,19 @@
         <v>102</v>
       </c>
       <c r="AR9" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="AS9" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="AS9" s="16" t="s">
-        <v>151</v>
-      </c>
       <c r="AT9" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="AU9" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV9" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW9" s="11" t="s">
@@ -3591,7 +3545,7 @@
         <v>107</v>
       </c>
       <c r="AY9" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X2RSBABA64</v>
       </c>
       <c r="AZ9" s="24" t="s">
@@ -3649,10 +3603,10 @@
         <v>74</v>
       </c>
       <c r="BR9" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS9" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS9" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT9" s="11" t="s">
         <v>74</v>
@@ -3661,7 +3615,6 @@
         <v>119</v>
       </c>
       <c r="BV9" s="31">
-        <f ca="1"/>
         <v>22924</v>
       </c>
       <c r="BW9" s="24">
@@ -3674,12 +3627,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" spans="1:77" s="33" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>189</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>190</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>72</v>
@@ -3694,13 +3647,13 @@
         <v>75</v>
       </c>
       <c r="G10" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="H10" s="14" t="s">
+      <c r="I10" s="15" t="s">
         <v>192</v>
-      </c>
-      <c r="I10" s="15" t="s">
-        <v>193</v>
       </c>
       <c r="J10" s="16" t="s">
         <v>79</v>
@@ -3709,7 +3662,7 @@
         <v>80</v>
       </c>
       <c r="L10" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M10" s="11" t="s">
@@ -3740,7 +3693,7 @@
         <v>80</v>
       </c>
       <c r="V10" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W10" s="16" t="s">
@@ -3750,7 +3703,7 @@
         <v>88</v>
       </c>
       <c r="Y10" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Z10" s="12" t="s">
         <v>90</v>
@@ -3774,11 +3727,11 @@
         <v>95</v>
       </c>
       <c r="AG10" s="23">
-        <f ca="1">V10+365</f>
+        <f>V10+365</f>
         <v>46090</v>
       </c>
       <c r="AH10" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AI10" s="16" t="s">
         <v>98</v>
@@ -3787,35 +3740,35 @@
         <v>99</v>
       </c>
       <c r="AK10" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL10" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM10" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN10" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO10" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP10" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AQ10" s="16" t="s">
         <v>102</v>
       </c>
       <c r="AR10" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="AS10" s="16" t="s">
         <v>178</v>
-      </c>
-      <c r="AS10" s="16" t="s">
-        <v>179</v>
       </c>
       <c r="AT10" s="11" t="s">
         <v>105</v>
@@ -3824,7 +3777,7 @@
         <v>106</v>
       </c>
       <c r="AV10" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW10" s="11" t="s">
@@ -3834,7 +3787,7 @@
         <v>107</v>
       </c>
       <c r="AY10" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X3RSBABA96</v>
       </c>
       <c r="AZ10" s="24" t="s">
@@ -3892,10 +3845,10 @@
         <v>74</v>
       </c>
       <c r="BR10" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS10" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS10" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT10" s="11" t="s">
         <v>74</v>
@@ -3904,7 +3857,6 @@
         <v>119</v>
       </c>
       <c r="BV10" s="31">
-        <f ca="1"/>
         <v>24042</v>
       </c>
       <c r="BW10" s="24">
@@ -3917,12 +3869,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>196</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>72</v>
@@ -3937,13 +3889,13 @@
         <v>75</v>
       </c>
       <c r="G11" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="H11" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="H11" s="14" t="s">
-        <v>198</v>
-      </c>
       <c r="I11" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J11" s="16" t="s">
         <v>79</v>
@@ -3952,7 +3904,7 @@
         <v>80</v>
       </c>
       <c r="L11" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M11" s="11" t="s">
@@ -3983,7 +3935,7 @@
         <v>80</v>
       </c>
       <c r="V11" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W11" s="16" t="s">
@@ -3993,13 +3945,13 @@
         <v>88</v>
       </c>
       <c r="Y11" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Z11" s="12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AA11" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB11" s="20" t="s">
         <v>92</v>
@@ -4014,14 +3966,14 @@
         <v>94</v>
       </c>
       <c r="AF11" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AG11" s="23">
-        <f ca="1">V11+365</f>
+        <f>V11+365</f>
         <v>46090</v>
       </c>
       <c r="AH11" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AI11" s="16" t="s">
         <v>98</v>
@@ -4030,26 +3982,26 @@
         <v>99</v>
       </c>
       <c r="AK11" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL11" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM11" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN11" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO11" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP11" s="16" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AQ11" s="16" t="s">
         <v>102</v>
@@ -4061,13 +4013,13 @@
         <v>104</v>
       </c>
       <c r="AT11" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AU11" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="AV11" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW11" s="11" t="s">
@@ -4077,7 +4029,7 @@
         <v>107</v>
       </c>
       <c r="AY11" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X1RSBABA70</v>
       </c>
       <c r="AZ11" s="24" t="s">
@@ -4135,10 +4087,10 @@
         <v>74</v>
       </c>
       <c r="BR11" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS11" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS11" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT11" s="11" t="s">
         <v>74</v>
@@ -4147,7 +4099,6 @@
         <v>119</v>
       </c>
       <c r="BV11" s="31">
-        <f ca="1"/>
         <v>74608</v>
       </c>
       <c r="BW11" s="24">
@@ -4160,12 +4111,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:77" s="33" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" ht="15.65" customHeight="1" spans="1:77" s="33" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>203</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>204</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>72</v>
@@ -4180,13 +4131,13 @@
         <v>75</v>
       </c>
       <c r="G12" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="H12" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="H12" s="14" t="s">
-        <v>206</v>
-      </c>
       <c r="I12" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J12" s="16" t="s">
         <v>79</v>
@@ -4195,7 +4146,7 @@
         <v>80</v>
       </c>
       <c r="L12" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M12" s="11" t="s">
@@ -4226,7 +4177,7 @@
         <v>80</v>
       </c>
       <c r="V12" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W12" s="16" t="s">
@@ -4239,7 +4190,7 @@
         <v>89</v>
       </c>
       <c r="Z12" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="AA12" s="12" t="s">
         <v>91</v>
@@ -4272,26 +4223,26 @@
         <v>99</v>
       </c>
       <c r="AK12" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL12" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM12" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN12" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN12" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO12" s="16" t="s">
         <v>100</v>
       </c>
       <c r="AP12" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AQ12" s="16" t="s">
         <v>102</v>
@@ -4303,13 +4254,13 @@
         <v>104</v>
       </c>
       <c r="AT12" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AU12" s="11" t="s">
         <v>96</v>
       </c>
       <c r="AV12" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW12" s="11" t="s">
@@ -4319,7 +4270,7 @@
         <v>107</v>
       </c>
       <c r="AY12" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X1RSBABA22</v>
       </c>
       <c r="AZ12" s="24" t="s">
@@ -4377,10 +4328,10 @@
         <v>74</v>
       </c>
       <c r="BR12" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS12" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS12" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT12" s="11" t="s">
         <v>74</v>
@@ -4389,7 +4340,6 @@
         <v>119</v>
       </c>
       <c r="BV12" s="31">
-        <f ca="1"/>
         <v>63937</v>
       </c>
       <c r="BW12" s="24">
@@ -4402,15 +4352,15 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B13" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="B13" s="35" t="s">
+      <c r="C13" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>73</v>
@@ -4428,7 +4378,7 @@
         <v>211</v>
       </c>
       <c r="I13" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>79</v>
@@ -4437,7 +4387,7 @@
         <v>80</v>
       </c>
       <c r="L13" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M13" s="11" t="s">
@@ -4468,7 +4418,7 @@
         <v>80</v>
       </c>
       <c r="V13" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W13" s="16" t="s">
@@ -4484,7 +4434,7 @@
         <v>213</v>
       </c>
       <c r="AA13" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB13" s="20" t="s">
         <v>92</v>
@@ -4502,7 +4452,7 @@
         <v>214</v>
       </c>
       <c r="AG13" s="23">
-        <f ca="1">V13+365</f>
+        <f>V13+365</f>
         <v>46090</v>
       </c>
       <c r="AH13" s="16" t="s">
@@ -4515,19 +4465,19 @@
         <v>216</v>
       </c>
       <c r="AK13" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL13" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM13" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN13" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO13" s="16" t="s">
@@ -4552,7 +4502,7 @@
         <v>96</v>
       </c>
       <c r="AV13" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW13" s="11" t="s">
@@ -4562,7 +4512,7 @@
         <v>107</v>
       </c>
       <c r="AY13" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X4RSBABA69</v>
       </c>
       <c r="AZ13" s="24" t="s">
@@ -4620,10 +4570,10 @@
         <v>74</v>
       </c>
       <c r="BR13" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS13" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS13" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT13" s="11" t="s">
         <v>74</v>
@@ -4632,7 +4582,6 @@
         <v>119</v>
       </c>
       <c r="BV13" s="31">
-        <f ca="1"/>
         <v>68634</v>
       </c>
       <c r="BW13" s="24">
@@ -4645,7 +4594,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="14" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>221</v>
       </c>
@@ -4671,7 +4620,7 @@
         <v>224</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J14" s="16" t="s">
         <v>79</v>
@@ -4680,7 +4629,7 @@
         <v>80</v>
       </c>
       <c r="L14" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M14" s="11" t="s">
@@ -4711,7 +4660,7 @@
         <v>80</v>
       </c>
       <c r="V14" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W14" s="16" t="s">
@@ -4757,20 +4706,20 @@
         <v>99</v>
       </c>
       <c r="AK14" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL14" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM14" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN14" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN14" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO14" s="16" t="s">
         <v>100</v>
@@ -4782,7 +4731,7 @@
         <v>102</v>
       </c>
       <c r="AR14" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="AS14" s="16" t="s">
         <v>227</v>
@@ -4794,7 +4743,7 @@
         <v>229</v>
       </c>
       <c r="AV14" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW14" s="11" t="s">
@@ -4804,7 +4753,7 @@
         <v>107</v>
       </c>
       <c r="AY14" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X6RSBABA45</v>
       </c>
       <c r="AZ14" s="24" t="s">
@@ -4862,10 +4811,10 @@
         <v>74</v>
       </c>
       <c r="BR14" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS14" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS14" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT14" s="11" t="s">
         <v>74</v>
@@ -4874,7 +4823,6 @@
         <v>119</v>
       </c>
       <c r="BV14" s="31">
-        <f ca="1"/>
         <v>54770</v>
       </c>
       <c r="BW14" s="24">
@@ -4887,7 +4835,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>230</v>
       </c>
@@ -4895,7 +4843,7 @@
         <v>231</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>72</v>
+        <v>209</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>73</v>
@@ -4913,7 +4861,7 @@
         <v>233</v>
       </c>
       <c r="I15" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>79</v>
@@ -4922,7 +4870,7 @@
         <v>80</v>
       </c>
       <c r="L15" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M15" s="11" t="s">
@@ -4953,7 +4901,7 @@
         <v>80</v>
       </c>
       <c r="V15" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W15" s="16" t="s">
@@ -4963,13 +4911,13 @@
         <v>88</v>
       </c>
       <c r="Y15" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="Z15" s="12" t="s">
         <v>213</v>
       </c>
       <c r="AA15" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB15" s="20" t="s">
         <v>92</v>
@@ -4987,11 +4935,11 @@
         <v>95</v>
       </c>
       <c r="AG15" s="23">
-        <f ca="1">V15+365</f>
+        <f>V15+365</f>
         <v>46090</v>
       </c>
       <c r="AH15" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="AI15" s="16" t="s">
         <v>98</v>
@@ -5000,19 +4948,19 @@
         <v>99</v>
       </c>
       <c r="AK15" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL15" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM15" s="24">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45725</v>
       </c>
       <c r="AN15" s="17">
-        <f t="shared" ca="1" si="5"/>
+        <f t="shared" si="5"/>
         <v>46090</v>
       </c>
       <c r="AO15" s="16" t="s">
@@ -5028,7 +4976,7 @@
         <v>218</v>
       </c>
       <c r="AS15" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AT15" s="11" t="s">
         <v>96</v>
@@ -5037,7 +4985,7 @@
         <v>96</v>
       </c>
       <c r="AV15" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW15" s="11" t="s">
@@ -5047,7 +4995,7 @@
         <v>107</v>
       </c>
       <c r="AY15" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X1RSBABA83</v>
       </c>
       <c r="AZ15" s="24" t="s">
@@ -5105,10 +5053,10 @@
         <v>74</v>
       </c>
       <c r="BR15" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS15" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS15" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT15" s="11" t="s">
         <v>74</v>
@@ -5117,7 +5065,6 @@
         <v>119</v>
       </c>
       <c r="BV15" s="31">
-        <f ca="1"/>
         <v>45160</v>
       </c>
       <c r="BW15" s="24">
@@ -5130,7 +5077,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:77" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" ht="15.65" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>235</v>
       </c>
@@ -5156,7 +5103,7 @@
         <v>238</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>79</v>
@@ -5165,7 +5112,7 @@
         <v>80</v>
       </c>
       <c r="L16" s="17">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45725</v>
       </c>
       <c r="M16" s="11" t="s">
@@ -5196,7 +5143,7 @@
         <v>80</v>
       </c>
       <c r="V16" s="17">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45725</v>
       </c>
       <c r="W16" s="16" t="s">
@@ -5212,7 +5159,7 @@
         <v>90</v>
       </c>
       <c r="AA16" s="12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="AB16" s="20" t="s">
         <v>92</v>
@@ -5227,7 +5174,7 @@
         <v>94</v>
       </c>
       <c r="AF16" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AG16" s="23" t="s">
         <v>96</v>
@@ -5242,20 +5189,20 @@
         <v>99</v>
       </c>
       <c r="AK16" s="24">
-        <f t="shared" ca="1" si="2"/>
+        <f t="shared" si="2"/>
         <v>45725</v>
       </c>
       <c r="AL16" s="24">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45725</v>
       </c>
       <c r="AM16" s="24">
-        <f t="shared" ca="1" si="4"/>
-        <v>45725</v>
-      </c>
-      <c r="AN16" s="17" t="str">
+        <f t="shared" si="4"/>
+        <v>45725</v>
+      </c>
+      <c r="AN16" s="17">
         <f t="shared" si="5"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AO16" s="16" t="s">
         <v>100</v>
@@ -5267,10 +5214,10 @@
         <v>102</v>
       </c>
       <c r="AR16" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="AS16" s="16" t="s">
         <v>178</v>
-      </c>
-      <c r="AS16" s="16" t="s">
-        <v>179</v>
       </c>
       <c r="AT16" s="11" t="s">
         <v>105</v>
@@ -5279,7 +5226,7 @@
         <v>106</v>
       </c>
       <c r="AV16" s="24">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>45776</v>
       </c>
       <c r="AW16" s="11" t="s">
@@ -5289,7 +5236,7 @@
         <v>107</v>
       </c>
       <c r="AY16" s="26" t="str">
-        <f t="shared" ca="1" si="7"/>
+        <f t="shared" si="7"/>
         <v>X8RSBABA86</v>
       </c>
       <c r="AZ16" s="24" t="s">
@@ -5347,10 +5294,10 @@
         <v>74</v>
       </c>
       <c r="BR16" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="BS16" s="11" t="s">
         <v>153</v>
-      </c>
-      <c r="BS16" s="11" t="s">
-        <v>154</v>
       </c>
       <c r="BT16" s="11" t="s">
         <v>74</v>
@@ -5359,7 +5306,6 @@
         <v>119</v>
       </c>
       <c r="BV16" s="31">
-        <f ca="1"/>
         <v>46967</v>
       </c>
       <c r="BW16" s="24">
@@ -5372,16 +5318,16 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.65" customHeight="1" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="C17" s="37" t="s">
-        <v>136</v>
+      <c r="C17" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AL17" s="24"/>
     </row>
-    <row r="18" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" ht="14.5" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G18" s="1" t="s">
         <v>241</v>
       </c>
@@ -5389,31 +5335,31 @@
         <v>242</v>
       </c>
     </row>
-    <row r="19" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="19" ht="14.5" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="C19" s="37" t="s">
-        <v>136</v>
+      <c r="C19" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="20" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="20" ht="14.5" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="C20" s="37" t="s">
-        <v>136</v>
+      <c r="C20" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="21" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="21" ht="14.5" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="C21" s="37" t="s">
-        <v>136</v>
+      <c r="C21" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="22" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="22" ht="14.5" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G22" s="1" t="s">
         <v>246</v>
       </c>
@@ -5421,15 +5367,15 @@
         <v>247</v>
       </c>
     </row>
-    <row r="23" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="23" ht="14.5" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="C23" s="37" t="s">
-        <v>136</v>
+      <c r="C23" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="24" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="24" ht="14.5" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G24" s="1" t="s">
         <v>249</v>
       </c>
@@ -5437,15 +5383,15 @@
         <v>250</v>
       </c>
     </row>
-    <row r="25" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="25" ht="14.5" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="C25" s="37" t="s">
-        <v>136</v>
+      <c r="C25" s="9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="26" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="26" ht="14.5" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G26" s="1" t="s">
         <v>252</v>
       </c>
@@ -5453,7 +5399,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="27" spans="2:54" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="27" ht="14.5" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
       <c r="G27" s="1" t="s">
         <v>254</v>
       </c>
@@ -5461,33 +5407,33 @@
         <v>255</v>
       </c>
     </row>
-    <row r="28" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="C28" s="37" t="s">
-        <v>136</v>
+      <c r="C28" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX28" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY28" s="38">
-        <f t="array" aca="1" ref="AY28:AY47" ca="1">_xlfn.RANDARRAY(20,1,1,9,TRUE)</f>
+      <c r="AY28" s="37">
+        <f t="array" ref="AY28:AY47">_xlfn.RANDARRAY(20,1,1,9,TRUE)</f>
         <v>7</v>
       </c>
       <c r="AZ28" s="26" t="s">
         <v>258</v>
       </c>
-      <c r="BA28" s="38">
-        <f t="array" aca="1" ref="BA28:BA47" ca="1">_xlfn.RANDARRAY(20,1,1,99,TRUE)</f>
+      <c r="BA28" s="37">
+        <f t="array" ref="BA28:BA47">_xlfn.RANDARRAY(20,1,1,99,TRUE)</f>
         <v>74</v>
       </c>
       <c r="BB28" s="1" t="str">
-        <f ca="1">AX28&amp;AY28&amp;AZ28&amp;BA28</f>
+        <f>AX28&amp;AY28&amp;AZ28&amp;BA28</f>
         <v>X7RSBABA74</v>
       </c>
     </row>
-    <row r="29" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G29" s="1" t="s">
         <v>259</v>
       </c>
@@ -5497,127 +5443,117 @@
       <c r="AX29" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY29" s="38">
-        <f ca="1"/>
+      <c r="AY29" s="37">
         <v>7</v>
       </c>
       <c r="AZ29" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA29" s="2">
-        <f ca="1"/>
         <v>15</v>
       </c>
       <c r="BB29" s="1" t="str">
-        <f t="shared" ref="BB29:BB53" ca="1" si="8">AX29&amp;AY29&amp;AZ29&amp;BA29</f>
+        <f t="shared" ref="BB29:BB53" si="8">AX29&amp;AY29&amp;AZ29&amp;BA29</f>
         <v>X7RSBABA15</v>
       </c>
     </row>
-    <row r="30" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="C30" s="37" t="s">
-        <v>136</v>
+      <c r="C30" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX30" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY30" s="38">
-        <f ca="1"/>
+      <c r="AY30" s="37">
         <v>8</v>
       </c>
       <c r="AZ30" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA30" s="2">
-        <f ca="1"/>
         <v>3</v>
       </c>
       <c r="BB30" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X8RSBABA3</v>
       </c>
     </row>
-    <row r="31" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="C31" s="37" t="s">
-        <v>136</v>
+      <c r="C31" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX31" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY31" s="38">
-        <f ca="1"/>
+      <c r="AY31" s="37">
         <v>9</v>
       </c>
       <c r="AZ31" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA31" s="2">
-        <f ca="1"/>
         <v>65</v>
       </c>
       <c r="BB31" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X9RSBABA65</v>
       </c>
     </row>
-    <row r="32" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C32" s="37" t="s">
-        <v>136</v>
+      <c r="C32" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX32" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY32" s="38">
-        <f ca="1"/>
+      <c r="AY32" s="37">
         <v>8</v>
       </c>
       <c r="AZ32" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA32" s="2">
-        <f ca="1"/>
         <v>96</v>
       </c>
       <c r="BB32" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X8RSBABA96</v>
       </c>
     </row>
-    <row r="33" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="C33" s="37" t="s">
-        <v>136</v>
+      <c r="C33" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX33" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY33" s="38">
-        <f ca="1"/>
+      <c r="AY33" s="37">
         <v>1</v>
       </c>
       <c r="AZ33" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA33" s="2">
-        <f ca="1"/>
         <v>20</v>
       </c>
       <c r="BB33" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X1RSBABA20</v>
       </c>
     </row>
-    <row r="34" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G34" s="1" t="s">
         <v>265</v>
       </c>
@@ -5627,23 +5563,21 @@
       <c r="AX34" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY34" s="38">
-        <f ca="1"/>
+      <c r="AY34" s="37">
         <v>2</v>
       </c>
       <c r="AZ34" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA34" s="2">
-        <f ca="1"/>
         <v>59</v>
       </c>
       <c r="BB34" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X2RSBABA59</v>
       </c>
     </row>
-    <row r="35" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G35" s="1" t="s">
         <v>267</v>
       </c>
@@ -5653,23 +5587,21 @@
       <c r="AX35" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY35" s="38">
-        <f ca="1"/>
+      <c r="AY35" s="37">
         <v>2</v>
       </c>
       <c r="AZ35" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA35" s="2">
-        <f ca="1"/>
         <v>64</v>
       </c>
       <c r="BB35" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X2RSBABA64</v>
       </c>
     </row>
-    <row r="36" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G36" s="1" t="s">
         <v>269</v>
       </c>
@@ -5679,23 +5611,21 @@
       <c r="AX36" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY36" s="38">
-        <f ca="1"/>
+      <c r="AY36" s="37">
         <v>3</v>
       </c>
       <c r="AZ36" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA36" s="2">
-        <f ca="1"/>
         <v>96</v>
       </c>
       <c r="BB36" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X3RSBABA96</v>
       </c>
     </row>
-    <row r="37" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G37" s="1" t="s">
         <v>271</v>
       </c>
@@ -5705,49 +5635,45 @@
       <c r="AX37" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY37" s="38">
-        <f ca="1"/>
+      <c r="AY37" s="37">
         <v>1</v>
       </c>
       <c r="AZ37" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA37" s="2">
-        <f ca="1"/>
         <v>70</v>
       </c>
       <c r="BB37" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X1RSBABA70</v>
       </c>
     </row>
-    <row r="38" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="C38" s="37" t="s">
-        <v>136</v>
+      <c r="C38" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX38" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY38" s="38">
-        <f ca="1"/>
+      <c r="AY38" s="37">
         <v>1</v>
       </c>
       <c r="AZ38" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA38" s="2">
-        <f ca="1"/>
         <v>22</v>
       </c>
       <c r="BB38" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X1RSBABA22</v>
       </c>
     </row>
-    <row r="39" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G39" s="1" t="s">
         <v>274</v>
       </c>
@@ -5757,23 +5683,21 @@
       <c r="AX39" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY39" s="38">
-        <f ca="1"/>
+      <c r="AY39" s="37">
         <v>4</v>
       </c>
       <c r="AZ39" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA39" s="2">
-        <f ca="1"/>
         <v>69</v>
       </c>
       <c r="BB39" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X4RSBABA69</v>
       </c>
     </row>
-    <row r="40" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G40" s="1" t="s">
         <v>276</v>
       </c>
@@ -5783,23 +5707,21 @@
       <c r="AX40" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY40" s="38">
-        <f ca="1"/>
+      <c r="AY40" s="37">
         <v>6</v>
       </c>
       <c r="AZ40" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA40" s="2">
-        <f ca="1"/>
         <v>45</v>
       </c>
       <c r="BB40" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X6RSBABA45</v>
       </c>
     </row>
-    <row r="41" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" ht="15.65" customHeight="1" spans="7:54" x14ac:dyDescent="0.25">
       <c r="G41" s="1" t="s">
         <v>278</v>
       </c>
@@ -5809,153 +5731,139 @@
       <c r="AX41" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY41" s="38">
-        <f ca="1"/>
+      <c r="AY41" s="37">
         <v>1</v>
       </c>
       <c r="AZ41" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA41" s="2">
-        <f ca="1"/>
         <v>83</v>
       </c>
       <c r="BB41" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X1RSBABA83</v>
       </c>
     </row>
-    <row r="42" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" ht="15.65" customHeight="1" spans="2:54" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="C42" s="37" t="s">
-        <v>136</v>
+      <c r="C42" s="9" t="s">
+        <v>209</v>
       </c>
       <c r="AX42" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY42" s="38">
-        <f ca="1"/>
+      <c r="AY42" s="37">
         <v>8</v>
       </c>
       <c r="AZ42" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA42" s="2">
-        <f ca="1"/>
         <v>86</v>
       </c>
       <c r="BB42" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X8RSBABA86</v>
       </c>
     </row>
-    <row r="43" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX43" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY43" s="38">
-        <f ca="1"/>
+      <c r="AY43" s="37">
         <v>7</v>
       </c>
       <c r="AZ43" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA43" s="2">
-        <f ca="1"/>
         <v>57</v>
       </c>
       <c r="BB43" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X7RSBABA57</v>
       </c>
     </row>
-    <row r="44" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX44" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY44" s="38">
-        <f ca="1"/>
+      <c r="AY44" s="37">
         <v>4</v>
       </c>
       <c r="AZ44" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA44" s="2">
-        <f ca="1"/>
         <v>87</v>
       </c>
       <c r="BB44" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X4RSBABA87</v>
       </c>
     </row>
-    <row r="45" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX45" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY45" s="38">
-        <f ca="1"/>
+      <c r="AY45" s="37">
         <v>1</v>
       </c>
       <c r="AZ45" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA45" s="2">
-        <f ca="1"/>
         <v>42</v>
       </c>
       <c r="BB45" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X1RSBABA42</v>
       </c>
     </row>
-    <row r="46" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX46" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY46" s="38">
-        <f ca="1"/>
+      <c r="AY46" s="37">
         <v>4</v>
       </c>
       <c r="AZ46" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA46" s="2">
-        <f ca="1"/>
         <v>67</v>
       </c>
       <c r="BB46" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X4RSBABA67</v>
       </c>
     </row>
-    <row r="47" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX47" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY47" s="38">
-        <f ca="1"/>
+      <c r="AY47" s="37">
         <v>3</v>
       </c>
       <c r="AZ47" s="26" t="s">
         <v>258</v>
       </c>
       <c r="BA47" s="2">
-        <f ca="1"/>
         <v>55</v>
       </c>
       <c r="BB47" s="1" t="str">
-        <f t="shared" ca="1" si="8"/>
+        <f t="shared" si="8"/>
         <v>X3RSBABA55</v>
       </c>
     </row>
-    <row r="48" spans="2:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX48" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY48" s="38"/>
+      <c r="AY48" s="37"/>
       <c r="AZ48" s="26" t="s">
         <v>258</v>
       </c>
@@ -5964,11 +5872,11 @@
         <v>XRSBABA</v>
       </c>
     </row>
-    <row r="49" spans="50:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX49" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY49" s="38"/>
+      <c r="AY49" s="37"/>
       <c r="AZ49" s="26" t="s">
         <v>258</v>
       </c>
@@ -5977,11 +5885,11 @@
         <v>XRSBABA</v>
       </c>
     </row>
-    <row r="50" spans="50:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX50" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="AY50" s="38"/>
+      <c r="AY50" s="37"/>
       <c r="AZ50" s="26" t="s">
         <v>258</v>
       </c>
@@ -5990,7 +5898,7 @@
         <v>XRSBABA</v>
       </c>
     </row>
-    <row r="51" spans="50:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX51" s="1" t="s">
         <v>257</v>
       </c>
@@ -6002,7 +5910,7 @@
         <v>XRSBABA</v>
       </c>
     </row>
-    <row r="52" spans="50:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" ht="15.65" customHeight="1" spans="50:54" x14ac:dyDescent="0.25">
       <c r="AX52" s="1" t="s">
         <v>257</v>
       </c>
@@ -6014,43 +5922,78 @@
         <v>XRSBABA</v>
       </c>
     </row>
-    <row r="53" spans="50:54" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="BB53" s="1" t="str">
+    <row r="53" ht="15.65" customHeight="1" spans="54:54" x14ac:dyDescent="0.25">
+      <c r="BB53" s="1">
         <f t="shared" si="8"/>
-        <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI10:AI16 W10:W16 U10:U16 R10:R16 K10:K16 BL10:BL16 AJ10:AJ12" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="15">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI10:AI16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2:AI16 W2:W16 U2:U16 R2:R16 K2:K16 BL2:BL16 AJ2:AJ12" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI2:AI16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ14:AJ16" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ12">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ14:AJ16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ12">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL10:BL16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K10:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R10:R16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="R2:R16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U10:U16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:U16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W10:W16">
+      <formula1>INDIRECT($E2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W16">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="T2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="T3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="T4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="T5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="T6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="T7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="T8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="T9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="T10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="T11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="T12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="T13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="T14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="T15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="T16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="T2" r:id="rId1"/>
+    <hyperlink ref="T3" r:id="rId2"/>
+    <hyperlink ref="T4" r:id="rId3"/>
+    <hyperlink ref="T5" r:id="rId4"/>
+    <hyperlink ref="T6" r:id="rId5"/>
+    <hyperlink ref="T7" r:id="rId6"/>
+    <hyperlink ref="T8" r:id="rId7"/>
+    <hyperlink ref="T9" r:id="rId8"/>
+    <hyperlink ref="T10" r:id="rId9"/>
+    <hyperlink ref="T11" r:id="rId10"/>
+    <hyperlink ref="T12" r:id="rId11"/>
+    <hyperlink ref="T13" r:id="rId12"/>
+    <hyperlink ref="T14" r:id="rId13"/>
+    <hyperlink ref="T15" r:id="rId14"/>
+    <hyperlink ref="T16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>